<commit_message>
Working on rebell again
</commit_message>
<xml_diff>
--- a/AmbermoonAdvanced.xlsx
+++ b/AmbermoonAdvanced.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="9"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Neue Daten Ep3" sheetId="1" state="visible" r:id="rId3"/>
@@ -1111,7 +1111,7 @@
     <t xml:space="preserve">408: Talked to S’Ebi once</t>
   </si>
   <si>
-    <t xml:space="preserve">409: Returned equip to S’Ebi</t>
+    <t xml:space="preserve">409: Talked to S’Ebi in hideout</t>
   </si>
   <si>
     <t xml:space="preserve">In Original all keywords from 0 to 114 are used.</t>

</xml_diff>